<commit_message>
copy rules and mapping
</commit_message>
<xml_diff>
--- a/config/sdt_templates/CUSEXTMI_API.xlsx
+++ b/config/sdt_templates/CUSEXTMI_API.xlsx
@@ -1,22 +1,22 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="27928"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29628"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://winpakltd-my.sharepoint.com/personal/warren_massey_winpak_com/Documents/data migration/toolset-v3/config/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\w10itasv\Documents\DataMigrationTool_v1.3\config\sdt_templates\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="430" documentId="8_{0D3EAE97-8E32-428E-8708-C4AAE827325D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{AD73B94F-5A38-493B-9BD9-19777DB812D3}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{A7982CDA-2BA8-4794-BE28-9A7A94FF3376}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="3120" yWindow="3120" windowWidth="21600" windowHeight="12645" xr2:uid="{9E07D46E-6301-46ED-BFAF-61A9F6943675}"/>
+    <workbookView xWindow="1560" yWindow="1560" windowWidth="21600" windowHeight="11235" xr2:uid="{9E07D46E-6301-46ED-BFAF-61A9F6943675}"/>
   </bookViews>
   <sheets>
     <sheet name="API_CUSEXTMI_AddFieldValue" sheetId="2" r:id="rId1"/>
     <sheet name="Sheet1" sheetId="1" r:id="rId2"/>
   </sheets>
-  <calcPr calcId="191029"/>
+  <calcPr calcId="191029" calcMode="manual"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -40,6 +40,7 @@
 <comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr">
   <authors>
     <author>Warren Massey</author>
+    <author>Vicente, Andres</author>
   </authors>
   <commentList>
     <comment ref="B2" authorId="0" shapeId="0" xr:uid="{492453BC-5698-449F-A7BD-6AB05DC8F23E}">
@@ -57,7 +58,7 @@
 Input/Output: IN_x000D_
 Position    : 16_x000D_
 Mandatory   : True_x000D_
-(Created: 2024-10-10 11:02:16 AM)</t>
+(Created: 2026-02-19 1:44:23 PM)</t>
         </r>
       </text>
     </comment>
@@ -76,7 +77,7 @@
 Input/Output: IN_x000D_
 Position    : 26_x000D_
 Mandatory   : False_x000D_
-(Created: 2024-10-10 11:02:16 AM)</t>
+(Created: 2026-02-19 1:44:24 PM)</t>
         </r>
       </text>
     </comment>
@@ -95,7 +96,7 @@
 Input/Output: IN_x000D_
 Position    : 56_x000D_
 Mandatory   : False_x000D_
-(Created: 2024-10-10 11:02:17 AM)</t>
+(Created: 2026-02-19 1:44:24 PM)</t>
         </r>
       </text>
     </comment>
@@ -114,7 +115,7 @@
 Input/Output: IN_x000D_
 Position    : 86_x000D_
 Mandatory   : False_x000D_
-(Created: 2024-10-10 11:02:17 AM)</t>
+(Created: 2026-02-19 1:44:24 PM)</t>
         </r>
       </text>
     </comment>
@@ -133,7 +134,7 @@
 Input/Output: IN_x000D_
 Position    : 116_x000D_
 Mandatory   : False_x000D_
-(Created: 2024-10-10 11:02:17 AM)</t>
+(Created: 2026-02-19 1:44:24 PM)</t>
         </r>
       </text>
     </comment>
@@ -152,7 +153,7 @@
 Input/Output: IN_x000D_
 Position    : 146_x000D_
 Mandatory   : False_x000D_
-(Created: 2024-10-10 11:02:18 AM)</t>
+(Created: 2026-02-19 1:44:24 PM)</t>
         </r>
       </text>
     </comment>
@@ -171,7 +172,7 @@
 Input/Output: IN_x000D_
 Position    : 176_x000D_
 Mandatory   : False_x000D_
-(Created: 2024-10-10 11:02:18 AM)</t>
+(Created: 2026-02-19 1:44:24 PM)</t>
         </r>
       </text>
     </comment>
@@ -190,7 +191,7 @@
 Input/Output: IN_x000D_
 Position    : 206_x000D_
 Mandatory   : False_x000D_
-(Created: 2024-10-10 11:02:18 AM)</t>
+(Created: 2026-02-19 1:44:24 PM)</t>
         </r>
       </text>
     </comment>
@@ -209,7 +210,7 @@
 Input/Output: IN_x000D_
 Position    : 236_x000D_
 Mandatory   : False_x000D_
-(Created: 2024-10-10 11:02:19 AM)</t>
+(Created: 2026-02-19 1:44:24 PM)</t>
         </r>
       </text>
     </comment>
@@ -228,7 +229,7 @@
 Input/Output: IN_x000D_
 Position    : 266_x000D_
 Mandatory   : False_x000D_
-(Created: 2024-10-10 11:02:20 AM)</t>
+(Created: 2026-02-19 1:44:24 PM)</t>
         </r>
       </text>
     </comment>
@@ -247,7 +248,7 @@
 Input/Output: IN_x000D_
 Position    : 296_x000D_
 Mandatory   : False_x000D_
-(Created: 2024-10-10 11:02:20 AM)</t>
+(Created: 2026-02-19 1:44:24 PM)</t>
         </r>
       </text>
     </comment>
@@ -266,7 +267,7 @@
 Input/Output: IN_x000D_
 Position    : 326_x000D_
 Mandatory   : False_x000D_
-(Created: 2024-10-10 11:02:21 AM)</t>
+(Created: 2026-02-19 1:44:25 PM)</t>
         </r>
       </text>
     </comment>
@@ -285,7 +286,7 @@
 Input/Output: IN_x000D_
 Position    : 356_x000D_
 Mandatory   : False_x000D_
-(Created: 2024-10-10 11:02:21 AM)</t>
+(Created: 2026-02-19 1:44:25 PM)</t>
         </r>
       </text>
     </comment>
@@ -304,7 +305,7 @@
 Input/Output: IN_x000D_
 Position    : 386_x000D_
 Mandatory   : False_x000D_
-(Created: 2024-10-10 11:02:25 AM)</t>
+(Created: 2026-02-19 1:44:25 PM)</t>
         </r>
       </text>
     </comment>
@@ -323,7 +324,7 @@
 Input/Output: IN_x000D_
 Position    : 416_x000D_
 Mandatory   : False_x000D_
-(Created: 2024-10-10 11:02:25 AM)</t>
+(Created: 2026-02-19 1:44:25 PM)</t>
         </r>
       </text>
     </comment>
@@ -342,7 +343,7 @@
 Input/Output: IN_x000D_
 Position    : 446_x000D_
 Mandatory   : False_x000D_
-(Created: 2024-10-10 11:02:26 AM)</t>
+(Created: 2026-02-19 1:44:25 PM)</t>
         </r>
       </text>
     </comment>
@@ -361,7 +362,7 @@
 Input/Output: IN_x000D_
 Position    : 476_x000D_
 Mandatory   : False_x000D_
-(Created: 2024-10-10 11:02:26 AM)</t>
+(Created: 2026-02-19 1:44:25 PM)</t>
         </r>
       </text>
     </comment>
@@ -380,7 +381,7 @@
 Input/Output: IN_x000D_
 Position    : 506_x000D_
 Mandatory   : False_x000D_
-(Created: 2024-10-10 11:02:26 AM)</t>
+(Created: 2026-02-19 1:44:25 PM)</t>
         </r>
       </text>
     </comment>
@@ -399,7 +400,7 @@
 Input/Output: IN_x000D_
 Position    : 536_x000D_
 Mandatory   : False_x000D_
-(Created: 2024-10-10 11:02:27 AM)</t>
+(Created: 2026-02-19 1:44:25 PM)</t>
         </r>
       </text>
     </comment>
@@ -418,7 +419,7 @@
 Input/Output: IN_x000D_
 Position    : 566_x000D_
 Mandatory   : False_x000D_
-(Created: 2024-10-10 11:02:27 AM)</t>
+(Created: 2026-02-19 1:44:25 PM)</t>
         </r>
       </text>
     </comment>
@@ -437,7 +438,7 @@
 Input/Output: IN_x000D_
 Position    : 587_x000D_
 Mandatory   : False_x000D_
-(Created: 2024-10-10 11:02:28 AM)</t>
+(Created: 2026-02-19 1:44:25 PM)</t>
         </r>
       </text>
     </comment>
@@ -456,7 +457,7 @@
 Input/Output: IN_x000D_
 Position    : 608_x000D_
 Mandatory   : False_x000D_
-(Created: 2024-10-10 11:02:28 AM)</t>
+(Created: 2026-02-19 1:44:25 PM)</t>
         </r>
       </text>
     </comment>
@@ -475,7 +476,7 @@
 Input/Output: IN_x000D_
 Position    : 629_x000D_
 Mandatory   : False_x000D_
-(Created: 2024-10-10 11:02:29 AM)</t>
+(Created: 2026-02-19 1:44:26 PM)</t>
         </r>
       </text>
     </comment>
@@ -494,7 +495,7 @@
 Input/Output: IN_x000D_
 Position    : 650_x000D_
 Mandatory   : False_x000D_
-(Created: 2024-10-10 11:02:29 AM)</t>
+(Created: 2026-02-19 1:44:26 PM)</t>
         </r>
       </text>
     </comment>
@@ -513,7 +514,7 @@
 Input/Output: IN_x000D_
 Position    : 671_x000D_
 Mandatory   : False_x000D_
-(Created: 2024-10-10 11:02:30 AM)</t>
+(Created: 2026-02-19 1:44:26 PM)</t>
         </r>
       </text>
     </comment>
@@ -532,7 +533,7 @@
 Input/Output: IN_x000D_
 Position    : 692_x000D_
 Mandatory   : False_x000D_
-(Created: 2024-10-10 11:02:33 AM)</t>
+(Created: 2026-02-19 1:44:26 PM)</t>
         </r>
       </text>
     </comment>
@@ -551,7 +552,7 @@
 Input/Output: IN_x000D_
 Position    : 713_x000D_
 Mandatory   : False_x000D_
-(Created: 2024-10-10 11:02:34 AM)</t>
+(Created: 2026-02-19 1:44:26 PM)</t>
         </r>
       </text>
     </comment>
@@ -570,7 +571,7 @@
 Input/Output: IN_x000D_
 Position    : 734_x000D_
 Mandatory   : False_x000D_
-(Created: 2024-10-10 11:02:34 AM)</t>
+(Created: 2026-02-19 1:44:26 PM)</t>
         </r>
       </text>
     </comment>
@@ -589,7 +590,7 @@
 Input/Output: IN_x000D_
 Position    : 755_x000D_
 Mandatory   : False_x000D_
-(Created: 2024-10-10 11:02:35 AM)</t>
+(Created: 2026-02-19 1:44:26 PM)</t>
         </r>
       </text>
     </comment>
@@ -608,7 +609,7 @@
 Input/Output: IN_x000D_
 Position    : 776_x000D_
 Mandatory   : False_x000D_
-(Created: 2024-10-10 11:02:35 AM)</t>
+(Created: 2026-02-19 1:44:26 PM)</t>
         </r>
       </text>
     </comment>
@@ -627,7 +628,7 @@
 Input/Output: IN_x000D_
 Position    : 777_x000D_
 Mandatory   : False_x000D_
-(Created: 2024-10-10 11:02:38 AM)</t>
+(Created: 2026-02-19 1:44:26 PM)</t>
         </r>
       </text>
     </comment>
@@ -646,538 +647,538 @@
 Input/Output: IN_x000D_
 Position    : 897_x000D_
 Mandatory   : False_x000D_
-(Created: 2024-10-10 11:02:40 AM)</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="B3" authorId="0" shapeId="0" xr:uid="{6B114002-E034-471E-BFAF-E63ADD5C1382}">
-      <text>
-        <r>
-          <rPr>
-            <b/>
-            <sz val="10"/>
-            <color indexed="81"/>
-            <rFont val="Courier New"/>
-            <family val="3"/>
-          </rPr>
-          <t>Control Codes: _x000D_
-T : Truncate to field length_x000D_
-U : Convert to Uppercase_x000D_
-B : Send blank values</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="C3" authorId="0" shapeId="0" xr:uid="{F55F5480-747B-41A7-A2BC-7EEE1798DC3C}">
-      <text>
-        <r>
-          <rPr>
-            <b/>
-            <sz val="10"/>
-            <color indexed="81"/>
-            <rFont val="Courier New"/>
-            <family val="3"/>
-          </rPr>
-          <t>Control Codes: _x000D_
-T : Truncate to field length_x000D_
-U : Convert to Uppercase_x000D_
-B : Send blank values</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="D3" authorId="0" shapeId="0" xr:uid="{CA275344-2AAA-4811-BB8B-19F74A968B86}">
-      <text>
-        <r>
-          <rPr>
-            <b/>
-            <sz val="10"/>
-            <color indexed="81"/>
-            <rFont val="Courier New"/>
-            <family val="3"/>
-          </rPr>
-          <t>Control Codes: _x000D_
-T : Truncate to field length_x000D_
-U : Convert to Uppercase_x000D_
-B : Send blank values</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="E3" authorId="0" shapeId="0" xr:uid="{B76F7081-4309-4EAD-BF8E-6F2471AD4142}">
-      <text>
-        <r>
-          <rPr>
-            <b/>
-            <sz val="10"/>
-            <color indexed="81"/>
-            <rFont val="Courier New"/>
-            <family val="3"/>
-          </rPr>
-          <t>Control Codes: _x000D_
-T : Truncate to field length_x000D_
-U : Convert to Uppercase_x000D_
-B : Send blank values</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="F3" authorId="0" shapeId="0" xr:uid="{181220A8-2ACA-45B7-9243-D96A2F33041F}">
-      <text>
-        <r>
-          <rPr>
-            <b/>
-            <sz val="10"/>
-            <color indexed="81"/>
-            <rFont val="Courier New"/>
-            <family val="3"/>
-          </rPr>
-          <t>Control Codes: _x000D_
-T : Truncate to field length_x000D_
-U : Convert to Uppercase_x000D_
-B : Send blank values</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="G3" authorId="0" shapeId="0" xr:uid="{24E4B816-948B-414F-B942-0FED61AD6917}">
-      <text>
-        <r>
-          <rPr>
-            <b/>
-            <sz val="10"/>
-            <color indexed="81"/>
-            <rFont val="Courier New"/>
-            <family val="3"/>
-          </rPr>
-          <t>Control Codes: _x000D_
-T : Truncate to field length_x000D_
-U : Convert to Uppercase_x000D_
-B : Send blank values</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="H3" authorId="0" shapeId="0" xr:uid="{94692E26-79D8-43CD-8E4C-4840B30416BD}">
-      <text>
-        <r>
-          <rPr>
-            <b/>
-            <sz val="10"/>
-            <color indexed="81"/>
-            <rFont val="Courier New"/>
-            <family val="3"/>
-          </rPr>
-          <t>Control Codes: _x000D_
-T : Truncate to field length_x000D_
-U : Convert to Uppercase_x000D_
-B : Send blank values</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="I3" authorId="0" shapeId="0" xr:uid="{83F73CD9-6D54-4AF4-BEA1-82F509EFBA53}">
-      <text>
-        <r>
-          <rPr>
-            <b/>
-            <sz val="10"/>
-            <color indexed="81"/>
-            <rFont val="Courier New"/>
-            <family val="3"/>
-          </rPr>
-          <t>Control Codes: _x000D_
-T : Truncate to field length_x000D_
-U : Convert to Uppercase_x000D_
-B : Send blank values</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="J3" authorId="0" shapeId="0" xr:uid="{952D6A91-9D88-4638-B53C-81D0E07CB7A6}">
-      <text>
-        <r>
-          <rPr>
-            <b/>
-            <sz val="10"/>
-            <color indexed="81"/>
-            <rFont val="Courier New"/>
-            <family val="3"/>
-          </rPr>
-          <t>Control Codes: _x000D_
-T : Truncate to field length_x000D_
-U : Convert to Uppercase_x000D_
-B : Send blank values</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="K3" authorId="0" shapeId="0" xr:uid="{DDA8F353-7A8D-4C47-A29A-C40EF9AB62BE}">
-      <text>
-        <r>
-          <rPr>
-            <b/>
-            <sz val="10"/>
-            <color indexed="81"/>
-            <rFont val="Courier New"/>
-            <family val="3"/>
-          </rPr>
-          <t>Control Codes: _x000D_
-T : Truncate to field length_x000D_
-U : Convert to Uppercase_x000D_
-B : Send blank values</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="L3" authorId="0" shapeId="0" xr:uid="{2220B24C-A67B-45DD-9C1B-47FE957EEEC0}">
-      <text>
-        <r>
-          <rPr>
-            <b/>
-            <sz val="10"/>
-            <color indexed="81"/>
-            <rFont val="Courier New"/>
-            <family val="3"/>
-          </rPr>
-          <t>Control Codes: _x000D_
-T : Truncate to field length_x000D_
-U : Convert to Uppercase_x000D_
-B : Send blank values</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="M3" authorId="0" shapeId="0" xr:uid="{3B2922B6-FFC3-41F3-9C22-4727D3332093}">
-      <text>
-        <r>
-          <rPr>
-            <b/>
-            <sz val="10"/>
-            <color indexed="81"/>
-            <rFont val="Courier New"/>
-            <family val="3"/>
-          </rPr>
-          <t>Control Codes: _x000D_
-T : Truncate to field length_x000D_
-U : Convert to Uppercase_x000D_
-B : Send blank values</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="N3" authorId="0" shapeId="0" xr:uid="{465B76FF-BDC7-422C-8F54-A420241DB45B}">
-      <text>
-        <r>
-          <rPr>
-            <b/>
-            <sz val="10"/>
-            <color indexed="81"/>
-            <rFont val="Courier New"/>
-            <family val="3"/>
-          </rPr>
-          <t>Control Codes: _x000D_
-T : Truncate to field length_x000D_
-U : Convert to Uppercase_x000D_
-B : Send blank values</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="O3" authorId="0" shapeId="0" xr:uid="{55BE56EE-95FB-48E9-8A0D-5D07076E4E06}">
-      <text>
-        <r>
-          <rPr>
-            <b/>
-            <sz val="10"/>
-            <color indexed="81"/>
-            <rFont val="Courier New"/>
-            <family val="3"/>
-          </rPr>
-          <t>Control Codes: _x000D_
-T : Truncate to field length_x000D_
-U : Convert to Uppercase_x000D_
-B : Send blank values</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="P3" authorId="0" shapeId="0" xr:uid="{808A2074-2300-4DFF-995C-B76A43A41860}">
-      <text>
-        <r>
-          <rPr>
-            <b/>
-            <sz val="10"/>
-            <color indexed="81"/>
-            <rFont val="Courier New"/>
-            <family val="3"/>
-          </rPr>
-          <t>Control Codes: _x000D_
-T : Truncate to field length_x000D_
-U : Convert to Uppercase_x000D_
-B : Send blank values</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="Q3" authorId="0" shapeId="0" xr:uid="{2F11C523-F4AB-4351-BEF9-8F798230C883}">
-      <text>
-        <r>
-          <rPr>
-            <b/>
-            <sz val="10"/>
-            <color indexed="81"/>
-            <rFont val="Courier New"/>
-            <family val="3"/>
-          </rPr>
-          <t>Control Codes: _x000D_
-T : Truncate to field length_x000D_
-U : Convert to Uppercase_x000D_
-B : Send blank values</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="R3" authorId="0" shapeId="0" xr:uid="{63B7381B-11B0-4756-A7F1-3FB13601A30B}">
-      <text>
-        <r>
-          <rPr>
-            <b/>
-            <sz val="10"/>
-            <color indexed="81"/>
-            <rFont val="Courier New"/>
-            <family val="3"/>
-          </rPr>
-          <t>Control Codes: _x000D_
-T : Truncate to field length_x000D_
-U : Convert to Uppercase_x000D_
-B : Send blank values</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="S3" authorId="0" shapeId="0" xr:uid="{10F0523A-C5B8-4317-81BB-0FE00355737B}">
-      <text>
-        <r>
-          <rPr>
-            <b/>
-            <sz val="10"/>
-            <color indexed="81"/>
-            <rFont val="Courier New"/>
-            <family val="3"/>
-          </rPr>
-          <t>Control Codes: _x000D_
-T : Truncate to field length_x000D_
-U : Convert to Uppercase_x000D_
-B : Send blank values</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="T3" authorId="0" shapeId="0" xr:uid="{9452588A-DB98-4A45-9BBE-71F70B313527}">
-      <text>
-        <r>
-          <rPr>
-            <b/>
-            <sz val="10"/>
-            <color indexed="81"/>
-            <rFont val="Courier New"/>
-            <family val="3"/>
-          </rPr>
-          <t>Control Codes: _x000D_
-T : Truncate to field length_x000D_
-U : Convert to Uppercase_x000D_
-B : Send blank values</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="U3" authorId="0" shapeId="0" xr:uid="{8C6E9500-AC2A-45E5-B122-90A712C6F6A5}">
-      <text>
-        <r>
-          <rPr>
-            <b/>
-            <sz val="10"/>
-            <color indexed="81"/>
-            <rFont val="Courier New"/>
-            <family val="3"/>
-          </rPr>
-          <t>Control Codes: _x000D_
-T : Truncate to field length_x000D_
-U : Convert to Uppercase_x000D_
-B : Send blank values</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="V3" authorId="0" shapeId="0" xr:uid="{B087A8F6-3B2B-46F5-B3A0-325017E0E814}">
-      <text>
-        <r>
-          <rPr>
-            <b/>
-            <sz val="10"/>
-            <color indexed="81"/>
-            <rFont val="Courier New"/>
-            <family val="3"/>
-          </rPr>
-          <t>Control Codes: _x000D_
-T : Truncate to field length_x000D_
-U : Convert to Uppercase_x000D_
-B : Send blank values</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="W3" authorId="0" shapeId="0" xr:uid="{78979A89-4BFE-4A08-831E-57C9D15A631D}">
-      <text>
-        <r>
-          <rPr>
-            <b/>
-            <sz val="10"/>
-            <color indexed="81"/>
-            <rFont val="Courier New"/>
-            <family val="3"/>
-          </rPr>
-          <t>Control Codes: _x000D_
-T : Truncate to field length_x000D_
-U : Convert to Uppercase_x000D_
-B : Send blank values</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="X3" authorId="0" shapeId="0" xr:uid="{2C48D566-FF4D-4876-9F32-E231288CC31B}">
-      <text>
-        <r>
-          <rPr>
-            <b/>
-            <sz val="10"/>
-            <color indexed="81"/>
-            <rFont val="Courier New"/>
-            <family val="3"/>
-          </rPr>
-          <t>Control Codes: _x000D_
-T : Truncate to field length_x000D_
-U : Convert to Uppercase_x000D_
-B : Send blank values</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="Y3" authorId="0" shapeId="0" xr:uid="{0AD173E5-DA39-475A-93FF-338AC80E9263}">
-      <text>
-        <r>
-          <rPr>
-            <b/>
-            <sz val="10"/>
-            <color indexed="81"/>
-            <rFont val="Courier New"/>
-            <family val="3"/>
-          </rPr>
-          <t>Control Codes: _x000D_
-T : Truncate to field length_x000D_
-U : Convert to Uppercase_x000D_
-B : Send blank values</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="Z3" authorId="0" shapeId="0" xr:uid="{4F0A9373-2A08-42F5-ACC2-1790F83B5987}">
-      <text>
-        <r>
-          <rPr>
-            <b/>
-            <sz val="10"/>
-            <color indexed="81"/>
-            <rFont val="Courier New"/>
-            <family val="3"/>
-          </rPr>
-          <t>Control Codes: _x000D_
-T : Truncate to field length_x000D_
-U : Convert to Uppercase_x000D_
-B : Send blank values</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="AA3" authorId="0" shapeId="0" xr:uid="{00F2BC1B-3E72-4230-8BD1-E246514BA5B0}">
-      <text>
-        <r>
-          <rPr>
-            <b/>
-            <sz val="10"/>
-            <color indexed="81"/>
-            <rFont val="Courier New"/>
-            <family val="3"/>
-          </rPr>
-          <t>Control Codes: _x000D_
-T : Truncate to field length_x000D_
-U : Convert to Uppercase_x000D_
-B : Send blank values</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="AB3" authorId="0" shapeId="0" xr:uid="{BE4EE7AE-169A-425C-84FF-985935D82569}">
-      <text>
-        <r>
-          <rPr>
-            <b/>
-            <sz val="10"/>
-            <color indexed="81"/>
-            <rFont val="Courier New"/>
-            <family val="3"/>
-          </rPr>
-          <t>Control Codes: _x000D_
-T : Truncate to field length_x000D_
-U : Convert to Uppercase_x000D_
-B : Send blank values</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="AC3" authorId="0" shapeId="0" xr:uid="{B503D8DA-52C5-4C72-9346-22AF72D43260}">
-      <text>
-        <r>
-          <rPr>
-            <b/>
-            <sz val="10"/>
-            <color indexed="81"/>
-            <rFont val="Courier New"/>
-            <family val="3"/>
-          </rPr>
-          <t>Control Codes: _x000D_
-T : Truncate to field length_x000D_
-U : Convert to Uppercase_x000D_
-B : Send blank values</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="AD3" authorId="0" shapeId="0" xr:uid="{F1635C37-43DF-4EDD-AF9F-C280740F87D6}">
-      <text>
-        <r>
-          <rPr>
-            <b/>
-            <sz val="10"/>
-            <color indexed="81"/>
-            <rFont val="Courier New"/>
-            <family val="3"/>
-          </rPr>
-          <t>Control Codes: _x000D_
-T : Truncate to field length_x000D_
-U : Convert to Uppercase_x000D_
-B : Send blank values</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="AE3" authorId="0" shapeId="0" xr:uid="{ABB09A7E-919D-4511-9490-7E30A1ADED93}">
-      <text>
-        <r>
-          <rPr>
-            <b/>
-            <sz val="10"/>
-            <color indexed="81"/>
-            <rFont val="Courier New"/>
-            <family val="3"/>
-          </rPr>
-          <t>Control Codes: _x000D_
-T : Truncate to field length_x000D_
-U : Convert to Uppercase_x000D_
-B : Send blank values</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="AF3" authorId="0" shapeId="0" xr:uid="{F9C619D1-F20B-4ECD-B293-BD37418AFA6C}">
-      <text>
-        <r>
-          <rPr>
-            <b/>
-            <sz val="10"/>
-            <color indexed="81"/>
-            <rFont val="Courier New"/>
-            <family val="3"/>
-          </rPr>
-          <t>Control Codes: _x000D_
-T : Truncate to field length_x000D_
-U : Convert to Uppercase_x000D_
-B : Send blank values</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="AG3" authorId="0" shapeId="0" xr:uid="{B9E7FA83-B125-43D8-AF5D-644D36288746}">
+(Created: 2026-02-19 1:44:27 PM)</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="B3" authorId="1" shapeId="0" xr:uid="{250664F8-CA72-4B8B-BEFB-963D98D3AE19}">
+      <text>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="10"/>
+            <color indexed="81"/>
+            <rFont val="Courier New"/>
+            <family val="3"/>
+          </rPr>
+          <t>Control Codes: _x000D_
+T : Truncate to field length_x000D_
+U : Convert to Uppercase_x000D_
+B : Send blank values</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="C3" authorId="1" shapeId="0" xr:uid="{93384E7C-93D8-4FF0-AF03-892499571D0C}">
+      <text>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="10"/>
+            <color indexed="81"/>
+            <rFont val="Courier New"/>
+            <family val="3"/>
+          </rPr>
+          <t>Control Codes: _x000D_
+T : Truncate to field length_x000D_
+U : Convert to Uppercase_x000D_
+B : Send blank values</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="D3" authorId="1" shapeId="0" xr:uid="{4F6097A4-CCBE-476E-8FBF-1CBCD9ECBA89}">
+      <text>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="10"/>
+            <color indexed="81"/>
+            <rFont val="Courier New"/>
+            <family val="3"/>
+          </rPr>
+          <t>Control Codes: _x000D_
+T : Truncate to field length_x000D_
+U : Convert to Uppercase_x000D_
+B : Send blank values</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="E3" authorId="1" shapeId="0" xr:uid="{6B467561-6CA7-448D-AFBC-14604E0B2187}">
+      <text>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="10"/>
+            <color indexed="81"/>
+            <rFont val="Courier New"/>
+            <family val="3"/>
+          </rPr>
+          <t>Control Codes: _x000D_
+T : Truncate to field length_x000D_
+U : Convert to Uppercase_x000D_
+B : Send blank values</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="F3" authorId="1" shapeId="0" xr:uid="{BEE4B0B7-6ACB-4B81-ADBA-3508A6E18BF4}">
+      <text>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="10"/>
+            <color indexed="81"/>
+            <rFont val="Courier New"/>
+            <family val="3"/>
+          </rPr>
+          <t>Control Codes: _x000D_
+T : Truncate to field length_x000D_
+U : Convert to Uppercase_x000D_
+B : Send blank values</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="G3" authorId="1" shapeId="0" xr:uid="{C44A04C6-3706-4025-88EA-64B0168FA3E8}">
+      <text>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="10"/>
+            <color indexed="81"/>
+            <rFont val="Courier New"/>
+            <family val="3"/>
+          </rPr>
+          <t>Control Codes: _x000D_
+T : Truncate to field length_x000D_
+U : Convert to Uppercase_x000D_
+B : Send blank values</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="H3" authorId="1" shapeId="0" xr:uid="{E1AE241C-5E83-4E78-A7E9-3A5EA84E3927}">
+      <text>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="10"/>
+            <color indexed="81"/>
+            <rFont val="Courier New"/>
+            <family val="3"/>
+          </rPr>
+          <t>Control Codes: _x000D_
+T : Truncate to field length_x000D_
+U : Convert to Uppercase_x000D_
+B : Send blank values</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="I3" authorId="1" shapeId="0" xr:uid="{D336B966-014E-4F80-96E3-03D67E30D730}">
+      <text>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="10"/>
+            <color indexed="81"/>
+            <rFont val="Courier New"/>
+            <family val="3"/>
+          </rPr>
+          <t>Control Codes: _x000D_
+T : Truncate to field length_x000D_
+U : Convert to Uppercase_x000D_
+B : Send blank values</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="J3" authorId="1" shapeId="0" xr:uid="{B22931A8-9799-4E74-98EB-3C08699E790B}">
+      <text>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="10"/>
+            <color indexed="81"/>
+            <rFont val="Courier New"/>
+            <family val="3"/>
+          </rPr>
+          <t>Control Codes: _x000D_
+T : Truncate to field length_x000D_
+U : Convert to Uppercase_x000D_
+B : Send blank values</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="K3" authorId="1" shapeId="0" xr:uid="{187E6688-E717-461F-8029-CA8B91B74EF5}">
+      <text>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="10"/>
+            <color indexed="81"/>
+            <rFont val="Courier New"/>
+            <family val="3"/>
+          </rPr>
+          <t>Control Codes: _x000D_
+T : Truncate to field length_x000D_
+U : Convert to Uppercase_x000D_
+B : Send blank values</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="L3" authorId="1" shapeId="0" xr:uid="{29F0DE9A-B3BC-45EB-9CD9-8390650D3E85}">
+      <text>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="10"/>
+            <color indexed="81"/>
+            <rFont val="Courier New"/>
+            <family val="3"/>
+          </rPr>
+          <t>Control Codes: _x000D_
+T : Truncate to field length_x000D_
+U : Convert to Uppercase_x000D_
+B : Send blank values</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="M3" authorId="1" shapeId="0" xr:uid="{38C0655A-2470-447B-83D1-53E35EF657F5}">
+      <text>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="10"/>
+            <color indexed="81"/>
+            <rFont val="Courier New"/>
+            <family val="3"/>
+          </rPr>
+          <t>Control Codes: _x000D_
+T : Truncate to field length_x000D_
+U : Convert to Uppercase_x000D_
+B : Send blank values</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="N3" authorId="1" shapeId="0" xr:uid="{DEEF5F5F-802C-42B4-A529-E5F02E9B1C26}">
+      <text>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="10"/>
+            <color indexed="81"/>
+            <rFont val="Courier New"/>
+            <family val="3"/>
+          </rPr>
+          <t>Control Codes: _x000D_
+T : Truncate to field length_x000D_
+U : Convert to Uppercase_x000D_
+B : Send blank values</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="O3" authorId="1" shapeId="0" xr:uid="{9E337EB4-A3E8-4FDE-ADAC-8DE2E7537255}">
+      <text>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="10"/>
+            <color indexed="81"/>
+            <rFont val="Courier New"/>
+            <family val="3"/>
+          </rPr>
+          <t>Control Codes: _x000D_
+T : Truncate to field length_x000D_
+U : Convert to Uppercase_x000D_
+B : Send blank values</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="P3" authorId="1" shapeId="0" xr:uid="{F07E8D1E-8128-46B3-A3D8-25F3F96166E9}">
+      <text>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="10"/>
+            <color indexed="81"/>
+            <rFont val="Courier New"/>
+            <family val="3"/>
+          </rPr>
+          <t>Control Codes: _x000D_
+T : Truncate to field length_x000D_
+U : Convert to Uppercase_x000D_
+B : Send blank values</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="Q3" authorId="1" shapeId="0" xr:uid="{45434F15-21A4-46FC-9A64-6C458367DD84}">
+      <text>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="10"/>
+            <color indexed="81"/>
+            <rFont val="Courier New"/>
+            <family val="3"/>
+          </rPr>
+          <t>Control Codes: _x000D_
+T : Truncate to field length_x000D_
+U : Convert to Uppercase_x000D_
+B : Send blank values</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="R3" authorId="1" shapeId="0" xr:uid="{DB91FCE4-349D-4F28-8CBD-29CF27258F97}">
+      <text>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="10"/>
+            <color indexed="81"/>
+            <rFont val="Courier New"/>
+            <family val="3"/>
+          </rPr>
+          <t>Control Codes: _x000D_
+T : Truncate to field length_x000D_
+U : Convert to Uppercase_x000D_
+B : Send blank values</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="S3" authorId="1" shapeId="0" xr:uid="{47FD1D5C-BD04-4648-8EFE-2D3F40063D5F}">
+      <text>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="10"/>
+            <color indexed="81"/>
+            <rFont val="Courier New"/>
+            <family val="3"/>
+          </rPr>
+          <t>Control Codes: _x000D_
+T : Truncate to field length_x000D_
+U : Convert to Uppercase_x000D_
+B : Send blank values</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="T3" authorId="1" shapeId="0" xr:uid="{AC221568-2142-463F-A5E1-50CDCE91886A}">
+      <text>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="10"/>
+            <color indexed="81"/>
+            <rFont val="Courier New"/>
+            <family val="3"/>
+          </rPr>
+          <t>Control Codes: _x000D_
+T : Truncate to field length_x000D_
+U : Convert to Uppercase_x000D_
+B : Send blank values</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="U3" authorId="1" shapeId="0" xr:uid="{3F166C1F-C16B-48BF-87FD-7F0F1EC60CEE}">
+      <text>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="10"/>
+            <color indexed="81"/>
+            <rFont val="Courier New"/>
+            <family val="3"/>
+          </rPr>
+          <t>Control Codes: _x000D_
+T : Truncate to field length_x000D_
+U : Convert to Uppercase_x000D_
+B : Send blank values</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="V3" authorId="1" shapeId="0" xr:uid="{240E7191-9567-456F-B8B8-B44ADE69D034}">
+      <text>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="10"/>
+            <color indexed="81"/>
+            <rFont val="Courier New"/>
+            <family val="3"/>
+          </rPr>
+          <t>Control Codes: _x000D_
+T : Truncate to field length_x000D_
+U : Convert to Uppercase_x000D_
+B : Send blank values</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="W3" authorId="1" shapeId="0" xr:uid="{AB2119CF-E278-4DDA-B29A-77ED806A9319}">
+      <text>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="10"/>
+            <color indexed="81"/>
+            <rFont val="Courier New"/>
+            <family val="3"/>
+          </rPr>
+          <t>Control Codes: _x000D_
+T : Truncate to field length_x000D_
+U : Convert to Uppercase_x000D_
+B : Send blank values</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="X3" authorId="1" shapeId="0" xr:uid="{DA9885DF-F3BC-4759-AAE4-8F0334AA38D6}">
+      <text>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="10"/>
+            <color indexed="81"/>
+            <rFont val="Courier New"/>
+            <family val="3"/>
+          </rPr>
+          <t>Control Codes: _x000D_
+T : Truncate to field length_x000D_
+U : Convert to Uppercase_x000D_
+B : Send blank values</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="Y3" authorId="1" shapeId="0" xr:uid="{67F154A7-4BEB-4D71-B745-79DCB831D51F}">
+      <text>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="10"/>
+            <color indexed="81"/>
+            <rFont val="Courier New"/>
+            <family val="3"/>
+          </rPr>
+          <t>Control Codes: _x000D_
+T : Truncate to field length_x000D_
+U : Convert to Uppercase_x000D_
+B : Send blank values</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="Z3" authorId="1" shapeId="0" xr:uid="{CBAB05A8-3E9C-47CE-AB7C-6437FB8121EA}">
+      <text>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="10"/>
+            <color indexed="81"/>
+            <rFont val="Courier New"/>
+            <family val="3"/>
+          </rPr>
+          <t>Control Codes: _x000D_
+T : Truncate to field length_x000D_
+U : Convert to Uppercase_x000D_
+B : Send blank values</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="AA3" authorId="1" shapeId="0" xr:uid="{F908AF0E-127C-48E0-A8BD-82B20F76EBF9}">
+      <text>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="10"/>
+            <color indexed="81"/>
+            <rFont val="Courier New"/>
+            <family val="3"/>
+          </rPr>
+          <t>Control Codes: _x000D_
+T : Truncate to field length_x000D_
+U : Convert to Uppercase_x000D_
+B : Send blank values</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="AB3" authorId="1" shapeId="0" xr:uid="{9A6D987E-443A-481C-B1BA-909131B2A361}">
+      <text>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="10"/>
+            <color indexed="81"/>
+            <rFont val="Courier New"/>
+            <family val="3"/>
+          </rPr>
+          <t>Control Codes: _x000D_
+T : Truncate to field length_x000D_
+U : Convert to Uppercase_x000D_
+B : Send blank values</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="AC3" authorId="1" shapeId="0" xr:uid="{60C22B7E-3127-45DB-9556-EF88E8F72A98}">
+      <text>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="10"/>
+            <color indexed="81"/>
+            <rFont val="Courier New"/>
+            <family val="3"/>
+          </rPr>
+          <t>Control Codes: _x000D_
+T : Truncate to field length_x000D_
+U : Convert to Uppercase_x000D_
+B : Send blank values</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="AD3" authorId="1" shapeId="0" xr:uid="{EF38C48A-5C71-46F9-BD78-97D95FBDB442}">
+      <text>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="10"/>
+            <color indexed="81"/>
+            <rFont val="Courier New"/>
+            <family val="3"/>
+          </rPr>
+          <t>Control Codes: _x000D_
+T : Truncate to field length_x000D_
+U : Convert to Uppercase_x000D_
+B : Send blank values</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="AE3" authorId="1" shapeId="0" xr:uid="{AC3E3C2E-FDB9-4F73-A645-24B5026930EC}">
+      <text>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="10"/>
+            <color indexed="81"/>
+            <rFont val="Courier New"/>
+            <family val="3"/>
+          </rPr>
+          <t>Control Codes: _x000D_
+T : Truncate to field length_x000D_
+U : Convert to Uppercase_x000D_
+B : Send blank values</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="AF3" authorId="1" shapeId="0" xr:uid="{95E4681B-68FF-4308-87D2-3C0064B372FF}">
+      <text>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="10"/>
+            <color indexed="81"/>
+            <rFont val="Courier New"/>
+            <family val="3"/>
+          </rPr>
+          <t>Control Codes: _x000D_
+T : Truncate to field length_x000D_
+U : Convert to Uppercase_x000D_
+B : Send blank values</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="AG3" authorId="1" shapeId="0" xr:uid="{A09B841C-2044-479E-9A41-58B79EF7130A}">
       <text>
         <r>
           <rPr>

</xml_diff>